<commit_message>
BRD-05 v2.0 sign-off and UX sets built; drop index updated
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-1_Transactional/BRD-05_Accounting_Disbursement_ACSL/04_BIBS_TestPlan_BRD-05_Accounting_Disbursement_ACSL_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-1_Transactional/BRD-05_Accounting_Disbursement_ACSL/04_BIBS_TestPlan_BRD-05_Accounting_Disbursement_ACSL_v2.0.xlsx
@@ -54178,7 +54178,7 @@
       <c r="L478" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-AC-01 Journals of the FRS.
-Fields in this order: 1 Status (Drop-down, mandatory N); 2 Batch no. (Text, mandatory N); 3 From / To (Date, mandatory N); 4 Inputter (Text, mandatory N); 5 Assignment (Drop-down, mandatory N); 6 Batch No. (Column, mandatory -); 7 Value Date (Column, mandatory -); 8 Type (Column, mandatory -); 9 Narration (Column, mandatory -); 10 Inputter / Assigned To / Authorizer (Column, mandatory -); 11 Amount (Column, mandatory -); 12 Status (Column, mandatory -); 13 Assign to (Drop-down, mandatory N); 14 Journals to post / Total debit / Selected but not pending (Display, mandatory -).
+Fields in this order: 1 Status (Drop-down, mandatory N); 2 Batch no. (Text, mandatory N); 3 From / To (Date, mandatory N); 4 Inputter (Text, mandatory N); 5 Assignment (Drop-down, mandatory N); 6 Batch No. (Column, mandatory -); 7 Value Date (Column, mandatory -); 8 Type (Column, mandatory -); 9 Narration (Column, mandatory -); 10 Inputter / Assigned To / Authorizer (Column, mandatory -); 11 Amount (Column, mandatory -); 12 Status (Column, mandatory -); 13 Assign to (Drop-down, mandatory N); 14 Journals to post, Total debit, Selected but not pending (Display, mandatory -).
 Actions: New Journal; Assign (n); Post Selected (n); Row.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -60750,24 +60750,23 @@
       <c r="L561" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-AC-321: "Added by the preparer"
-MSG-AC-325: "Account &lt;code&gt; is a heading" (ACSL_ACCOUNT_NOT_POSTABLE)
-MSG-AC-326: "Account &lt;code&gt; is not in the chart" (ACSL_ACCOUNT_UNKNOWN)
-MSG-AC-327: "A ledger component (&lt;components&gt;) needs the invoice it corrects" (ACSL_COMPONENT_INVALID)
-MSG-AC-328: "A correction needs at least two lines and equal debits (&lt;to plain string&gt;) and credits (&lt;to plain string&gt;)" (ACSL_CORRECTION_UNBALANCED)
-MSG-AC-329: "Describe the correction" (ACSL_DESCRIPTION_REQUIRED)
-MSG-AC-330: "A correction is reviewed by someone other than its preparer" (ACSL_FOUR_EYES)
-MSG-AC-331: "The approver of a correction is not its maker" (ACSL_FOUR_EYES)
-MSG-AC-332: "Invoice &lt;invoice&gt; is not in the ledger" (ACSL_INVOICE_UNKNOWN)
-MSG-AC-333: "Invoice &lt;no&gt; is not in the ledger" (ACSL_INVOICE_UNKNOWN)
-MSG-AC-334: "Journal &lt;batch no&gt; not found" (ACSL_JOURNAL_UNKNOWN)
-MSG-AC-335: "Every line needs a GL account" (ACSL_LINE_INVALID)
-MSG-AC-336: "Every line needs a side and a positive amount with two decimals" (ACSL_LINE_INVALID)
-MSG-AC-337: "Journal &lt;batch no&gt; has no line &lt;line no&gt;" (ACSL_LINE_UNKNOWN)
-MSG-AC-338: "The company has no branch" (ACSL_NO_BRANCH)
-MSG-AC-339: "Control account &lt;code&gt; needs the sub-ledger party" (ACSL_PARTY_REQUIRED)
-MSG-AC-340: "Party &lt;code&gt; of a correction line is not maintained" (ACSL_PARTY_UNKNOWN)
-MSG-AC-341: "A correction has at most 200 lines" (ACSL_TOO_MANY_LINES)</t>
+MSG-AC-324: "Account &lt;code&gt; is a heading" (ACSL_ACCOUNT_NOT_POSTABLE)
+MSG-AC-325: "Account &lt;code&gt; is not in the chart" (ACSL_ACCOUNT_UNKNOWN)
+MSG-AC-326: "A ledger component (&lt;components&gt;) needs the invoice it corrects" (ACSL_COMPONENT_INVALID)
+MSG-AC-327: "A correction needs at least two lines and equal debits (&lt;to plain string&gt;) and credits (&lt;to plain string&gt;)" (ACSL_CORRECTION_UNBALANCED)
+MSG-AC-328: "Describe the correction" (ACSL_DESCRIPTION_REQUIRED)
+MSG-AC-329: "A correction is reviewed by someone other than its preparer" (ACSL_FOUR_EYES)
+MSG-AC-330: "The approver of a correction is not its maker" (ACSL_FOUR_EYES)
+MSG-AC-331: "Invoice &lt;invoice&gt; is not in the ledger" (ACSL_INVOICE_UNKNOWN)
+MSG-AC-332: "Invoice &lt;no&gt; is not in the ledger" (ACSL_INVOICE_UNKNOWN)
+MSG-AC-333: "Journal &lt;batch no&gt; not found" (ACSL_JOURNAL_UNKNOWN)
+MSG-AC-334: "Every line needs a GL account" (ACSL_LINE_INVALID)
+MSG-AC-335: "Every line needs a side and a positive amount with two decimals" (ACSL_LINE_INVALID)
+MSG-AC-336: "Journal &lt;batch no&gt; has no line &lt;line no&gt;" (ACSL_LINE_UNKNOWN)
+MSG-AC-337: "The company has no branch" (ACSL_NO_BRANCH)
+MSG-AC-338: "Control account &lt;code&gt; needs the sub-ledger party" (ACSL_PARTY_REQUIRED)
+MSG-AC-339: "Party &lt;code&gt; of a correction line is not maintained" (ACSL_PARTY_UNKNOWN)
+MSG-AC-340: "A correction has at most 200 lines" (ACSL_TOO_MANY_LINES)</t>
         </is>
       </c>
       <c r="M561" s="12" t="inlineStr">
@@ -60842,11 +60841,11 @@
       <c r="L562" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-AC-344: "The file does not follow the layout '&lt;name&gt;'; missing column(s): &lt;missing&gt;" (ACSL_SOA_LAYOUT_MISMATCH)
-MSG-AC-345: "No SOA layout is configured" (ACSL_SOA_NO_LAYOUT)
-MSG-AC-346: "Give the insurer and the covered period of the statement" (ACSL_SOA_PERIOD)
-MSG-AC-347: "The covered period ends before it starts" (ACSL_SOA_PERIOD)
-MSG-AC-348: "An SOA upload has at most &lt;max&gt; rows" (ACSL_SOA_TOO_LARGE)</t>
+MSG-AC-343: "The file does not follow the layout '&lt;name&gt;'; missing column(s): &lt;missing&gt;" (ACSL_SOA_LAYOUT_MISMATCH)
+MSG-AC-344: "No SOA layout is configured" (ACSL_SOA_NO_LAYOUT)
+MSG-AC-345: "Give the insurer and the covered period of the statement" (ACSL_SOA_PERIOD)
+MSG-AC-346: "The covered period ends before it starts" (ACSL_SOA_PERIOD)
+MSG-AC-347: "An SOA upload has at most &lt;max&gt; rows" (ACSL_SOA_TOO_LARGE)</t>
         </is>
       </c>
       <c r="M562" s="12" t="inlineStr">
@@ -60921,7 +60920,7 @@
       <c r="L563" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-AC-351: "The file must be at most 10 MB" (ACSL_SOA_TOO_LARGE)</t>
+MSG-AC-350: "The file must be at most 10 MB" (ACSL_SOA_TOO_LARGE)</t>
         </is>
       </c>
       <c r="M563" s="12" t="inlineStr">
@@ -60996,7 +60995,7 @@
       <c r="L564" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-AC-355: "Give the sub-ledger, and the components (Operations ledger) or document types (open items)" (ACSL_GLSL_SETTING)</t>
+MSG-AC-354: "Give the sub-ledger, and the components (Operations ledger) or document types (open items)" (ACSL_GLSL_SETTING)</t>
         </is>
       </c>
       <c r="M564" s="12" t="inlineStr">
@@ -61059,10 +61058,10 @@
       <c r="L565" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-AC-356: "The account becomes active and can be posted to."
-MSG-AC-357: "The bank account change takes effect."
-MSG-AC-358: "The request is closed without creating a payee."
-MSG-AC-359: "The status change is sent for authorisation."</t>
+MSG-AC-355: "The account becomes active and can be posted to."
+MSG-AC-356: "The bank account change takes effect."
+MSG-AC-357: "The request is closed without creating a payee."
+MSG-AC-358: "The status change is sent for authorisation."</t>
         </is>
       </c>
       <c r="M565" s="12" t="inlineStr">
@@ -61137,8 +61136,8 @@
       <c r="L566" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-AC-360: "&lt;Column&gt; '&lt;value&gt;' is not a valid &lt;number, date (yyyy-mm-dd), Y/N value&gt;"
-MSG-AC-361: "&lt;Column&gt; is mandatory"</t>
+MSG-AC-359: "&lt;Column&gt; '&lt;value&gt;' is not a valid &lt;number, date (yyyy-mm-dd), Y/N value&gt;"
+MSG-AC-360: "&lt;Column&gt; is mandatory"</t>
         </is>
       </c>
       <c r="M566" s="12" t="inlineStr">
@@ -61213,12 +61212,12 @@
       <c r="L567" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-AC-362: "&lt;header&gt; must be one of &lt;details&gt;"
-MSG-AC-363: "Account &lt;code&gt; already exists"
-MSG-AC-364: "Account Code may hold digits, capital letters, '.' and '-' only"
-MSG-AC-365: "Currencies must be three-letter codes separated by commas"
-MSG-AC-366: "Enter the account code of a top-level account"
-MSG-AC-367: "Parent &lt;parent&gt; is neither an account nor an earlier row of the file"</t>
+MSG-AC-361: "&lt;header&gt; must be one of &lt;details&gt;"
+MSG-AC-362: "Account &lt;code&gt; already exists"
+MSG-AC-363: "Account Code may hold digits, capital letters, '.' and '-' only"
+MSG-AC-364: "Currencies must be three-letter codes separated by commas"
+MSG-AC-365: "Enter the account code of a top-level account"
+MSG-AC-366: "Parent &lt;parent&gt; is neither an account nor an earlier row of the file"</t>
         </is>
       </c>
       <c r="M567" s="12" t="inlineStr">
@@ -61293,9 +61292,9 @@
       <c r="L568" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-AC-368: "The amount must be positive"
-MSG-AC-369: "The currency must be a 3-letter code"
-MSG-AC-371: "Unknown disbursement type &lt;type&gt;"</t>
+MSG-AC-367: "The amount must be positive"
+MSG-AC-368: "The currency must be a 3-letter code"
+MSG-AC-370: "Unknown disbursement type &lt;type&gt;"</t>
         </is>
       </c>
       <c r="M568" s="12" t="inlineStr">
@@ -61370,8 +61369,8 @@
       <c r="L569" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-AC-370: "The default mode must be one of the allowed modes"
-MSG-AC-372: "Unknown mode of payment: &lt;message&gt;"</t>
+MSG-AC-369: "The default mode must be one of the allowed modes"
+MSG-AC-371: "Unknown mode of payment: &lt;message&gt;"</t>
         </is>
       </c>
       <c r="M569" s="12" t="inlineStr">
@@ -61434,13 +61433,13 @@
       <c r="L570" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-AC-373: "You are not permitted to perform this action" (ACCESS_DENIED)
-MSG-AC-374: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
-MSG-AC-375: "The system could not complete the request. Try again; if it continues, contact support with the reference." (INTERNAL_ERROR)
-MSG-AC-376: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
-MSG-AC-377: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
-MSG-AC-378: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
-MSG-AC-379: "Invalid request" (VALIDATION_FAILED)</t>
+MSG-AC-372: "You are not permitted to perform this action" (ACCESS_DENIED)
+MSG-AC-373: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
+MSG-AC-374: "The system could not complete the request. Try again; if it continues, contact support with the reference." (INTERNAL_ERROR)
+MSG-AC-375: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
+MSG-AC-376: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
+MSG-AC-377: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
+MSG-AC-378: "Invalid request" (VALIDATION_FAILED)</t>
         </is>
       </c>
       <c r="M570" s="12" t="inlineStr">

</xml_diff>